<commit_message>
Sweep: model qty (N(n)), BACK + ANGLE-ALT/SIDE-ALT views, * CSV variable block
- parseSweepName: support quantity-in-brackets model tokens, e.g. 46(2) = model
  46 cloned twice, expanded into the nums array.
- New view types: BACK (-180, like HEAD rotated 180), ANGLE-ALT (-35) and
  SIDE-ALT (-90), tested before their base keywords.
- camera_coordinates.csv restructured: one shared "* (ALL VARIANTS)" block
  defines each view once; OTTOMAN is the only per-variant override (others
  inherit). lookupCameraCoords scoring made lexicographic (viewtype specificity
  primary, exact variant tiebreaker) so * inheritance is robust.
- OTTOMAN non-top rows: cleared Y=0 so the camera pulls back on -Y again
  (was rendering overhead like a top shot).
- TOP RATIO 0.33; DETAIL rotation -15 across variants.
- Add build_mse.ms helper to encrypt current script into a shareable output\.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/EXCEL/EXCEL FILE.xlsx
+++ b/EXCEL/EXCEL FILE.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\SWEEP SCRIPT\EXCEL\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A0036A8D-AF53-4CA8-890A-05727744CB13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C9A6C9D-77E0-43E2-88DD-483B822026EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="41400" yWindow="3000" windowWidth="28800" windowHeight="15370" xr2:uid="{95237670-869A-4140-B156-ED85E052E114}"/>
+    <workbookView xWindow="8480" yWindow="4090" windowWidth="18790" windowHeight="15370" xr2:uid="{95237670-869A-4140-B156-ED85E052E114}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -602,7 +602,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D1ACE807-3E7A-4790-B7F1-31A13D478A76}">
-  <dimension ref="A1:A64"/>
+  <dimension ref="A1:A65"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="33.08984375" bestFit="1" customWidth="1"/>
@@ -928,6 +928,13 @@
         <v>63</v>
       </c>
     </row>
+    <row r="65" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>87214-08-TOP-SW-AGR</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>